<commit_message>
thêm chức năng thẻ tab theo dõi xe tổng thể
</commit_message>
<xml_diff>
--- a/docs/bảng lắp.xlsx
+++ b/docs/bảng lắp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ki5\line_follower_robot_arm\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5295B44-FF64-4BB6-AC36-49104C95C3E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E159A29-2947-47B8-95BD-DA4BD22E989F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A5366B0F-4077-4238-95FA-ECA0532C2CE2}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>Linh kiện</t>
   </si>
@@ -148,6 +148,18 @@
   </si>
   <si>
     <t>RIGHT</t>
+  </si>
+  <si>
+    <t>dưới cam</t>
+  </si>
+  <si>
+    <t>trên vàng</t>
+  </si>
+  <si>
+    <t>dưới nâu</t>
+  </si>
+  <si>
+    <t>trên đỏ</t>
   </si>
 </sst>
 </file>
@@ -578,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BC95E1-ADEA-48A9-8B1F-8595292FC68F}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
@@ -759,7 +771,7 @@
       </c>
       <c r="D16" s="5"/>
     </row>
-    <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
       <c r="B17" s="5" t="s">
         <v>25</v>
@@ -769,7 +781,7 @@
       </c>
       <c r="D17" s="5"/>
     </row>
-    <row r="18" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
       <c r="B18" s="5" t="s">
         <v>26</v>
@@ -779,7 +791,7 @@
       </c>
       <c r="D18" s="5"/>
     </row>
-    <row r="19" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
       <c r="B19" s="5" t="s">
         <v>27</v>
@@ -789,7 +801,7 @@
       </c>
       <c r="D19" s="5"/>
     </row>
-    <row r="20" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="5" t="s">
         <v>33</v>
@@ -798,8 +810,11 @@
       <c r="D20" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="5" t="s">
         <v>34</v>
@@ -808,8 +823,11 @@
       <c r="D21" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
       <c r="B22" s="5" t="s">
         <v>35</v>
@@ -818,8 +836,11 @@
       <c r="D22" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="21" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
       <c r="B23" s="5" t="s">
         <v>36</v>
@@ -827,6 +848,9 @@
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
         <v>38</v>
+      </c>
+      <c r="E23" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>